<commit_message>
add iclr 25 papers & fix some errors
</commit_message>
<xml_diff>
--- a/Paper Collections.xlsx
+++ b/Paper Collections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\Awesome-Interpretable-Network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF8EA06-F475-4FF4-8E0F-49F4CE09D495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9391DC61-F6D0-4431-9465-DFA4364A9E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4752" yWindow="120" windowWidth="24564" windowHeight="16152" firstSheet="1" activeTab="6" xr2:uid="{DC4A0462-C16D-4CCA-9144-463242733AF6}"/>
+    <workbookView xWindow="4752" yWindow="120" windowWidth="24564" windowHeight="16152" firstSheet="1" activeTab="9" xr2:uid="{DC4A0462-C16D-4CCA-9144-463242733AF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Attribution-based" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="425">
   <si>
     <t>EMNLP</t>
   </si>
@@ -741,9 +741,6 @@
     <t>[TECHS: Temporal logical graph networks for explainable extrapolation reasoning](https://doi.org/10.18653/v1/2023.acl-long.71)</t>
   </si>
   <si>
-    <t>[SIG: Efficient Self-Interpretable Graph Neural Network for Continuous-time Dynamic Graphs](https://doi.org/10.48550/arXiv.2405.19062)</t>
-  </si>
-  <si>
     <t>[How Interpretable Are Interpretable Graph Neural Networks?](https://openreview.net/forum?id=F3G2udCF3Q)</t>
   </si>
   <si>
@@ -1167,9 +1164,6 @@
     <t>[Code](https://github.com/wuyxin/dir-gnn)</t>
   </si>
   <si>
-    <t>[Code](https://github.com/2024sig/sig)</t>
-  </si>
-  <si>
     <t>[Code](https://github.com/Wangyuwen0627/GIP-Framework)</t>
   </si>
   <si>
@@ -1264,6 +1258,66 @@
   </si>
   <si>
     <t>[Code](https://github.com/fawazsammani/nlxgpt)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/yangji721/SeSRDQN)</t>
+  </si>
+  <si>
+    <t>[Counterfactual Concept Bottleneck Models](https://openreview.net/forum?id=w7pMjyjsKN)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/gabriele-dominici/Counterfactual-CBM)</t>
+  </si>
+  <si>
+    <t>[Causal Concept Graph Models: Beyond Causal Opacity in Deep Learning](https://openreview.net/forum?id=lmKJ1b6PaL)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/gabriele-dominici/CausalCGM)</t>
+  </si>
+  <si>
+    <t>[Concept Bottleneck Large Language Models](https://openreview.net/forum?id=RC5FPYVQaH)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/Trustworthy-ML-Lab/CB-LLMs)</t>
+  </si>
+  <si>
+    <t>[Concept Bottleneck Language Models For protein design](https://openreview.net/forum?id=Yt9CFhOOFe)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/prescient-design/lobster)</t>
+  </si>
+  <si>
+    <t>[Restyling Unsupervised Concept Based Interpretable Networks with Generative Models](https://openreview.net/forum?id=CexatBp6rx)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/GnRlLeclerc/VisCoIN)</t>
+  </si>
+  <si>
+    <t>[Adaptive Concept Bottleneck for Foundation Models](https://openreview.net/forum?id=8sfc8MwG5v)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/jihyechoi77/CONDA)</t>
+  </si>
+  <si>
+    <t>[Lucid{PPN}: Unambiguous Prototypical Parts Network for User-centric Interpretable Computer Vision](https://openreview.net/forum?id=BM9qfolt6p)</t>
+  </si>
+  <si>
+    <t>[Intrinsic User-Centric Interpretability through Global Mixture of Experts](https://openreview.net/forum?id=wDcunIOAOk)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/epfl-ml4ed/interpretcc)</t>
+  </si>
+  <si>
+    <t>[Factor Graph-based Interpretable Neural Networks](https://openreview.net/forum?id=10DtLPsdro)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/yushuowiki/AGAIN)</t>
+  </si>
+  <si>
+    <t>[From {GNN}s to Trees: Multi-Granular Interpretability for Graph Neural Networks](https://openreview.net/forum?id=KEUPk0wXXe)</t>
+  </si>
+  <si>
+    <t>[Code](https://github.com/dutyj2020/TIF)</t>
   </si>
 </sst>
 </file>
@@ -1641,7 +1695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D597EF-B3E6-4DE3-AD47-33AB211D4C6C}">
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="89.109375" style="2" customWidth="1"/>
@@ -1662,7 +1716,7 @@
         <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1676,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1690,7 +1744,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1704,7 +1758,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1718,7 +1772,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1732,7 +1786,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1746,7 +1800,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1760,7 +1814,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1774,7 +1828,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1788,7 +1842,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1802,7 +1856,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1816,7 +1870,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1830,7 +1884,7 @@
         <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1844,7 +1898,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1858,7 +1912,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1872,7 +1926,7 @@
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1886,7 +1940,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1900,7 +1954,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1914,7 +1968,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -1928,7 +1982,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1942,7 +1996,7 @@
         <v>6</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1956,7 +2010,7 @@
         <v>0</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -1970,7 +2024,7 @@
         <v>13</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1984,7 +2038,7 @@
         <v>1</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1998,7 +2052,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2012,7 +2066,7 @@
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2026,7 +2080,7 @@
         <v>7</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2040,7 +2094,7 @@
         <v>7</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2054,7 +2108,7 @@
         <v>14</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2068,7 +2122,7 @@
         <v>55</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2082,7 +2136,7 @@
         <v>3</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2096,7 +2150,7 @@
         <v>58</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2110,7 +2164,7 @@
         <v>2</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2124,7 +2178,7 @@
         <v>7</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2138,7 +2192,7 @@
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2152,7 +2206,7 @@
         <v>14</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2166,7 +2220,7 @@
         <v>3</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2180,7 +2234,7 @@
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2194,7 +2248,7 @@
         <v>2</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2208,7 +2262,7 @@
         <v>1</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2222,7 +2276,7 @@
         <v>2</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2236,7 +2290,7 @@
         <v>12</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2250,7 +2304,7 @@
         <v>6</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2264,7 +2318,7 @@
         <v>15</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2278,7 +2332,7 @@
         <v>5</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2292,7 +2346,7 @@
         <v>8</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -2306,7 +2360,7 @@
         <v>4</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -2320,7 +2374,7 @@
         <v>12</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -2334,7 +2388,7 @@
         <v>6</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -2348,7 +2402,7 @@
         <v>3</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -2362,7 +2416,7 @@
         <v>1</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -2376,7 +2430,7 @@
         <v>2</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -2390,7 +2444,7 @@
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -2404,7 +2458,7 @@
         <v>9</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -2418,7 +2472,7 @@
         <v>5</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -2432,7 +2486,7 @@
         <v>18</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -2446,7 +2500,7 @@
         <v>1</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -2460,7 +2514,7 @@
         <v>2</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -2474,7 +2528,7 @@
         <v>5</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -2488,7 +2542,7 @@
         <v>2</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -2502,7 +2556,7 @@
         <v>2</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -2516,7 +2570,7 @@
         <v>6</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -2530,7 +2584,7 @@
         <v>90</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2544,7 +2598,7 @@
         <v>17</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -2558,7 +2612,7 @@
         <v>6</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -2572,7 +2626,7 @@
         <v>3</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -2586,7 +2640,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -2600,7 +2654,7 @@
         <v>16</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -2614,7 +2668,7 @@
         <v>2</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -2628,7 +2682,7 @@
         <v>13</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2642,7 +2696,7 @@
         <v>1</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -2656,7 +2710,7 @@
         <v>3</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -2670,7 +2724,7 @@
         <v>9</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -2684,7 +2738,7 @@
         <v>12</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -2698,7 +2752,7 @@
         <v>1</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -2712,7 +2766,7 @@
         <v>1</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -2726,7 +2780,7 @@
         <v>2</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -2740,7 +2794,7 @@
         <v>13</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -2754,7 +2808,7 @@
         <v>2</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -2768,7 +2822,7 @@
         <v>2</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -2782,7 +2836,7 @@
         <v>3</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -2796,7 +2850,7 @@
         <v>2</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -2810,7 +2864,7 @@
         <v>9</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -2824,7 +2878,7 @@
         <v>3</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -2838,7 +2892,21 @@
         <v>10</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B86" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -2869,12 +2937,12 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B2" s="3">
         <v>2018</v>
@@ -2883,7 +2951,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2897,7 +2965,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2911,7 +2979,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2925,7 +2993,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2939,7 +3007,7 @@
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2953,7 +3021,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2967,12 +3035,12 @@
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B9" s="3">
         <v>2023</v>
@@ -2981,12 +3049,12 @@
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B10" s="3">
         <v>2023</v>
@@ -2995,12 +3063,12 @@
         <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B11" s="3">
         <v>2023</v>
@@ -3009,7 +3077,7 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -3020,15 +3088,15 @@
         <v>2024</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D12" t="s">
-        <v>262</v>
+        <v>405</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B13" s="3">
         <v>2024</v>
@@ -3037,7 +3105,7 @@
         <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -3051,12 +3119,12 @@
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B15" s="3">
         <v>2024</v>
@@ -3065,7 +3133,7 @@
         <v>6</v>
       </c>
       <c r="D15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -3079,7 +3147,7 @@
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -3093,12 +3161,12 @@
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B18" s="3">
         <v>2024</v>
@@ -3107,12 +3175,12 @@
         <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B19" s="3">
         <v>2024</v>
@@ -3121,7 +3189,7 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -3151,7 +3219,7 @@
         <v>25</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3165,7 +3233,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -3179,7 +3247,7 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3193,7 +3261,7 @@
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -3207,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -3221,7 +3289,7 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -3235,7 +3303,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -3249,7 +3317,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -3263,7 +3331,7 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -3277,7 +3345,7 @@
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -3291,7 +3359,7 @@
         <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -3305,7 +3373,7 @@
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -3315,17 +3383,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B132377C-8AE1-442B-A5C4-1805A89C2262}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="77.33203125" customWidth="1"/>
+    <col min="1" max="1" width="77.33203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" style="3" customWidth="1"/>
     <col min="3" max="3" width="31" style="3" customWidth="1"/>
     <col min="4" max="4" width="41.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -3335,11 +3403,11 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>123</v>
       </c>
       <c r="B2" s="3">
@@ -3349,11 +3417,11 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>124</v>
       </c>
       <c r="B3" s="3">
@@ -3363,11 +3431,11 @@
         <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B4" s="3">
@@ -3377,11 +3445,11 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>125</v>
       </c>
       <c r="B5" s="3">
@@ -3391,11 +3459,11 @@
         <v>126</v>
       </c>
       <c r="D5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B6" s="3">
@@ -3405,11 +3473,11 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>127</v>
       </c>
       <c r="B7" s="3">
@@ -3419,11 +3487,11 @@
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>128</v>
       </c>
       <c r="B8" s="3">
@@ -3433,11 +3501,11 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>129</v>
       </c>
       <c r="B9" s="3">
@@ -3447,11 +3515,11 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>130</v>
       </c>
       <c r="B10" s="3">
@@ -3461,11 +3529,11 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>131</v>
       </c>
       <c r="B11" s="3">
@@ -3475,11 +3543,11 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" t="s">
+      <c r="A12" s="2" t="s">
         <v>132</v>
       </c>
       <c r="B12" s="3">
@@ -3489,11 +3557,11 @@
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>133</v>
       </c>
       <c r="B13" s="3">
@@ -3503,11 +3571,11 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>134</v>
       </c>
       <c r="B14" s="3">
@@ -3517,11 +3585,11 @@
         <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>135</v>
       </c>
       <c r="B15" s="3">
@@ -3531,11 +3599,11 @@
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>136</v>
       </c>
       <c r="B16" s="3">
@@ -3545,11 +3613,11 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>137</v>
       </c>
       <c r="B17" s="3">
@@ -3559,11 +3627,11 @@
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>138</v>
       </c>
       <c r="B18" s="3">
@@ -3573,11 +3641,11 @@
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>139</v>
       </c>
       <c r="B19" s="3">
@@ -3587,11 +3655,11 @@
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" t="s">
+      <c r="A20" s="2" t="s">
         <v>140</v>
       </c>
       <c r="B20" s="3">
@@ -3601,11 +3669,11 @@
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>141</v>
       </c>
       <c r="B21" s="3">
@@ -3615,11 +3683,11 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>142</v>
       </c>
       <c r="B22" s="3">
@@ -3629,11 +3697,11 @@
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>143</v>
       </c>
       <c r="B23" s="3">
@@ -3643,11 +3711,11 @@
         <v>5</v>
       </c>
       <c r="D23" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>144</v>
       </c>
       <c r="B24" s="3">
@@ -3657,11 +3725,11 @@
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>145</v>
       </c>
       <c r="B25" s="3">
@@ -3671,11 +3739,96 @@
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>262</v>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B26" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B27" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B28" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D28" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B29" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D29" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B30" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D30" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B31" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D31" t="s">
+        <v>417</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3702,7 +3855,7 @@
         <v>25</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3716,7 +3869,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -3730,7 +3883,7 @@
         <v>14</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3744,7 +3897,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -3758,7 +3911,7 @@
         <v>20</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -3772,7 +3925,7 @@
         <v>14</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -3786,7 +3939,7 @@
         <v>5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -3800,7 +3953,7 @@
         <v>5</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -3814,7 +3967,7 @@
         <v>10</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -3828,7 +3981,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -3842,7 +3995,7 @@
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -3856,7 +4009,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -3870,7 +4023,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -3884,7 +4037,7 @@
         <v>3</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -3898,7 +4051,7 @@
         <v>20</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -3912,7 +4065,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -3926,7 +4079,7 @@
         <v>21</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -3940,7 +4093,7 @@
         <v>2</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -3954,7 +4107,7 @@
         <v>6</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -3968,7 +4121,7 @@
         <v>2</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -3982,11 +4135,22 @@
         <v>17</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>262</v>
+        <v>405</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="5"/>
+      <c r="A22" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B22" s="6">
+        <v>2025</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4015,7 +4179,7 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4029,7 +4193,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -4043,7 +4207,7 @@
         <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -4057,7 +4221,7 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -4071,7 +4235,7 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -4085,7 +4249,7 @@
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -4099,7 +4263,7 @@
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -4113,7 +4277,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -4127,7 +4291,7 @@
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -4141,7 +4305,7 @@
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -4155,7 +4319,7 @@
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -4169,7 +4333,7 @@
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -4183,7 +4347,7 @@
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -4197,7 +4361,7 @@
         <v>175</v>
       </c>
       <c r="D14" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -4211,7 +4375,7 @@
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -4225,7 +4389,7 @@
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -4239,7 +4403,7 @@
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -4253,7 +4417,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -4267,7 +4431,7 @@
         <v>13</v>
       </c>
       <c r="D19" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -4281,7 +4445,7 @@
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -4295,7 +4459,7 @@
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -4309,7 +4473,7 @@
         <v>4</v>
       </c>
       <c r="D22" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -4323,7 +4487,7 @@
         <v>12</v>
       </c>
       <c r="D23" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -4337,7 +4501,7 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -4351,7 +4515,7 @@
         <v>175</v>
       </c>
       <c r="D25" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -4365,7 +4529,7 @@
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -4379,7 +4543,7 @@
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -4393,7 +4557,7 @@
         <v>2</v>
       </c>
       <c r="D28" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -4423,7 +4587,7 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4437,7 +4601,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -4451,7 +4615,7 @@
         <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -4465,7 +4629,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -4479,7 +4643,7 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -4493,7 +4657,7 @@
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -4507,7 +4671,7 @@
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -4521,7 +4685,7 @@
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -4535,7 +4699,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -4549,7 +4713,7 @@
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -4563,7 +4727,7 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -4577,7 +4741,7 @@
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -4591,7 +4755,7 @@
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -4605,7 +4769,7 @@
         <v>20</v>
       </c>
       <c r="D14" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -4619,7 +4783,7 @@
         <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -4633,7 +4797,7 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -4663,7 +4827,7 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4677,7 +4841,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -4691,7 +4855,7 @@
         <v>197</v>
       </c>
       <c r="D3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -4705,7 +4869,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -4719,7 +4883,7 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -4733,7 +4897,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -4747,7 +4911,7 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -4761,7 +4925,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -4775,7 +4939,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -4789,7 +4953,7 @@
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -4803,7 +4967,7 @@
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -4817,7 +4981,7 @@
         <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -4831,7 +4995,7 @@
         <v>175</v>
       </c>
       <c r="D13" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -4845,7 +5009,7 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -4859,7 +5023,7 @@
         <v>207</v>
       </c>
       <c r="D15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -4873,7 +5037,7 @@
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -4887,7 +5051,7 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -4901,7 +5065,7 @@
         <v>211</v>
       </c>
       <c r="D18" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -4915,7 +5079,7 @@
         <v>2</v>
       </c>
       <c r="D19" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -4929,7 +5093,7 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -4943,7 +5107,7 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -4957,7 +5121,7 @@
         <v>197</v>
       </c>
       <c r="D22" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -4971,7 +5135,7 @@
         <v>15</v>
       </c>
       <c r="D23" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -4985,7 +5149,7 @@
         <v>6</v>
       </c>
       <c r="D24" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -4999,7 +5163,7 @@
         <v>0</v>
       </c>
       <c r="D25" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -5013,7 +5177,7 @@
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -5027,7 +5191,7 @@
         <v>211</v>
       </c>
       <c r="D27" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -5041,7 +5205,7 @@
         <v>7</v>
       </c>
       <c r="D28" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -5055,7 +5219,7 @@
         <v>7</v>
       </c>
       <c r="D29" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -5065,10 +5229,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61AFBF71-C3F3-454D-A049-13E0D1909E3B}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="70.77734375" customWidth="1"/>
+    <col min="1" max="1" width="85.88671875" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" style="3" customWidth="1"/>
     <col min="3" max="3" width="20.33203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="35.6640625" customWidth="1"/>
@@ -5085,7 +5249,7 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -5099,7 +5263,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -5113,7 +5277,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -5127,7 +5291,7 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -5141,7 +5305,7 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -5155,7 +5319,7 @@
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -5169,7 +5333,7 @@
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -5183,7 +5347,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -5197,7 +5361,7 @@
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -5211,7 +5375,7 @@
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -5225,7 +5389,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -5239,7 +5403,7 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -5253,7 +5417,7 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -5267,40 +5431,40 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>232</v>
+        <v>110</v>
       </c>
       <c r="B15" s="3">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>374</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B16" s="3">
         <v>2024</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>262</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B17" s="3">
         <v>2024</v>
@@ -5314,7 +5478,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B18" s="3">
         <v>2024</v>
@@ -5328,16 +5492,16 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>232</v>
       </c>
       <c r="B19" s="3">
         <v>2024</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>313</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -5348,10 +5512,10 @@
         <v>2024</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D20" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -5362,10 +5526,10 @@
         <v>2024</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>262</v>
+        <v>373</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -5376,10 +5540,10 @@
         <v>2024</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>375</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -5390,29 +5554,29 @@
         <v>2024</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>237</v>
+        <v>105</v>
       </c>
       <c r="B24" s="3">
         <v>2024</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>237</v>
       </c>
       <c r="B25" s="3">
         <v>2024</v>
@@ -5421,7 +5585,7 @@
         <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -5432,24 +5596,38 @@
         <v>2024</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>239</v>
+        <v>421</v>
       </c>
       <c r="B27" s="3">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" t="s">
-        <v>262</v>
+        <v>422</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>423</v>
+      </c>
+      <c r="B28" s="3">
+        <v>2025</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D28" t="s">
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -5479,12 +5657,12 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B2" s="3">
         <v>2019</v>
@@ -5493,12 +5671,12 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B3" s="3">
         <v>2019</v>
@@ -5507,12 +5685,12 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B4" s="3">
         <v>2019</v>
@@ -5521,12 +5699,12 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B5" s="3">
         <v>2020</v>
@@ -5535,12 +5713,12 @@
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B6" s="3">
         <v>2020</v>
@@ -5549,12 +5727,12 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B7" s="3">
         <v>2021</v>
@@ -5563,7 +5741,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -5577,12 +5755,12 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B9" s="3">
         <v>2023</v>
@@ -5591,7 +5769,7 @@
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -5605,12 +5783,12 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B11" s="3">
         <v>2023</v>
@@ -5619,12 +5797,12 @@
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B12" s="3">
         <v>2023</v>
@@ -5633,7 +5811,7 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -5647,7 +5825,7 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -5661,12 +5839,12 @@
         <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B15" s="3">
         <v>2023</v>
@@ -5675,12 +5853,12 @@
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B16" s="3">
         <v>2024</v>
@@ -5689,7 +5867,7 @@
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>